<commit_message>
docs(suivi): MAJ Excel - chat v2 (#216, #219, #220, #307, Phase 2 #156, #194 partiel) + suivi technique
Suivi technique : temps réel, carte produit, anti-contournement, facture
vendeur, push FCM à faire ; sauvegardes externalisées marquées réalisées
(2026-09-11).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -8807,14 +8807,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F229" s="23" t="inlineStr">
-        <is>
-          <t>🟡 Partiel</t>
+      <c r="F229" s="21" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G229" s="22" t="inlineStr">
         <is>
-          <t>Itération 7 — limité au cadre du litige</t>
+          <t>Chat v2 (2026-09-18) : fils acheteur-boutique en temps réel, fiche produit depuis l'article, photos/PDF, messages vocaux, accusé « Vu », blocage des coordonnées</t>
         </is>
       </c>
     </row>
@@ -8912,14 +8912,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F232" s="23" t="inlineStr">
-        <is>
-          <t>🟡 Partiel</t>
+      <c r="F232" s="21" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="G232" s="22" t="inlineStr">
         <is>
-          <t>Itération 7 — fil de litige conservé</t>
+          <t>Conversations conservées (/compte/messages, /vendeur/messages) ; 200 derniers messages par fil</t>
         </is>
       </c>
     </row>
@@ -8954,7 +8954,7 @@
       </c>
       <c r="G233" s="22" t="inlineStr">
         <is>
-          <t>Itération 9 — messages de litige notifiés aux autres parties</t>
+          <t>Itération 9 (litiges) + messagerie : notification in-app, email si le destinataire est hors ligne, badges non-lus en temps réel</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="G325" s="22" t="inlineStr">
         <is>
-          <t>Itération 9 — fil de litige</t>
+          <t>Itération 9 (litiges) + messagerie acheteur-boutique (in-app + email si hors ligne)</t>
         </is>
       </c>
     </row>
@@ -17145,7 +17145,12 @@
       </c>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Chat v2 : photos (JPG/PNG/WebP), PDF et messages vocaux, 10 Mo max, Storage privé</t>
         </is>
       </c>
     </row>
@@ -18305,9 +18310,14 @@
           <t>Basse</t>
         </is>
       </c>
-      <c r="F209" s="4" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F209" s="23" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Blocage automatique des coordonnées + surveillance admin (lecture journalisée des fils) ; signalement manuel par l'utilisateur à venir</t>
         </is>
       </c>
     </row>
@@ -42289,7 +42299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="26" min="1" max="1"/>
@@ -42302,7 +42312,7 @@
     <row r="1">
       <c r="A1" s="37" t="inlineStr">
         <is>
-          <t>SUIVI TECHNIQUE - TRAVAUX HORS CAHIER DES CHARGES (MAJ 2026-07-10)</t>
+          <t>SUIVI TECHNIQUE - TRAVAUX HORS CAHIER DES CHARGES (MAJ 2026-09-18)</t>
         </is>
       </c>
     </row>
@@ -42377,7 +42387,6 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -42398,7 +42407,6 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -42469,7 +42477,6 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -42590,7 +42597,6 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -42636,7 +42642,6 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -42732,7 +42737,6 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -42828,7 +42832,6 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -42849,7 +42852,6 @@
           <t>✅ Réalisé</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -42972,7 +42974,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>À publier dans la console Firebase (fournies)</t>
+          <t>À publier dans la console Firebase (fournies) ; nouveau dossier chat/ (messagerie) à publier en console</t>
         </is>
       </c>
     </row>
@@ -43045,7 +43047,6 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -43058,17 +43059,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Sauvegardes externalisées chiffrées (Backblaze B2 / Object Storage)</t>
+          <t>Sauvegardes externalisées chiffrées (hors VPS)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Obligatoire avant argent réel</t>
+          <t>Dump chiffré (age) vers le bucket GCS, 30 jours, test de restauration validé (2026-09-11)</t>
         </is>
       </c>
     </row>
@@ -43122,7 +43123,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" s="26">
       <c r="A36" t="n">
         <v>34</v>
       </c>
@@ -43141,7 +43142,131 @@
           <t>À faire</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+    </row>
+    <row r="37" s="26">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Messagerie</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Temps réel Postgres LISTEN/NOTIFY + SSE : messages, « Vu », « en train d'écrire », badges</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Lot 1 flux acheteur-vendeur (2026-09-18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" s="26">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Messagerie</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Carte « Se renseigner sur ce produit » depuis une fiche produit</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Lot 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" s="26">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Modération</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Anti-contournement : blocage des coordonnées (messages, fiches, boutique, profil) + mise sous surveillance</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Lot 1 - page admin Surveillance, lecture des fils journalisée</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" s="26">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Facture PDF exemplaire vendeur sans le téléphone de l'acheteur</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Lot 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" s="26">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Messagerie</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Notifications push (FCM) des nouveaux messages</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Clé Web Push à générer dans la console Firebase</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - Ma liste / favoris (Phase 2 #6, #7, #63), historique (Phase 3 #2), baisse de prix (#75 partiel) + suivi technique
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -12468,7 +12468,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>« Ma liste » (lot 2, 2026-09-18) : cœur sur la fiche et sur toutes les cartes produit, une liste par compte, prix à l'ajout mémorisé</t>
         </is>
       </c>
     </row>
@@ -12498,7 +12503,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Page /compte/liste : produits gardés, « Tout ajouter au panier », ruptures et produits retirés signalés</t>
         </is>
       </c>
     </row>
@@ -14254,7 +14264,12 @@
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>« Vus récemment » : 50 dernières fiches consultées par compte, affichées dans Ma liste</t>
         </is>
       </c>
     </row>
@@ -20379,7 +20394,12 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Historique des fiches consultées (« Vus récemment »), effaçable par l'utilisateur</t>
         </is>
       </c>
     </row>
@@ -22764,12 +22784,19 @@
           <t>Basse</t>
         </is>
       </c>
-      <c r="F94" s="6" t="inlineStr">
-        <is>
-          <t>À faire</t>
-        </is>
-      </c>
-    </row>
+      <c r="F94" s="23" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Badge « Prix en baisse » dans Ma liste (prix à l'ajout mémorisé) ; notification à venir</t>
+        </is>
+      </c>
+    </row>
+    <row r="95"/>
+    <row r="96"/>
     <row r="97" ht="16.3" customHeight="1" s="26">
       <c r="A97" s="33" t="inlineStr">
         <is>
@@ -42299,7 +42326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="26" min="1" max="1"/>
@@ -43268,6 +43295,81 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Parcours d'achat</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Fiche produit : Acheter maintenant / Ajouter au panier / Discuter / Ma liste + barre d'actions fixe sur mobile</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Lot 2 flux acheteur-vendeur (2026-09-18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Parcours d'achat</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Achat direct : commande d'un seul article sans toucher au panier, reprise après connexion</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Lot 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Vendeur</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Nombre d'acheteurs ayant chaque produit dans leur liste (Mes produits)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Lot 2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - devis/bons de commande (Phase 2 #77), frais de service et remboursements (#114, #125, #254, #271) + suivi technique
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -5264,7 +5264,7 @@
       </c>
       <c r="G122" s="22" t="inlineStr">
         <is>
-          <t>Itération 5 — commission 5 % au versement vendeur</t>
+          <t>Itération 5 — commission 5 % au versement vendeur ; lot 3 (2026-09-18) : frais de service acheteur 1 % (non remboursables) + frais Mobile Money répercutés à la recharge, paramétrables</t>
         </is>
       </c>
     </row>
@@ -5649,7 +5649,7 @@
       </c>
       <c r="G133" s="22" t="inlineStr">
         <is>
-          <t>Itérations 5-8 — annulation, litige et intervention admin</t>
+          <t>Itérations 5-8 — annulation, litige et intervention admin ; depuis le lot 3, hors frais de service (non remboursables)</t>
         </is>
       </c>
     </row>
@@ -10151,7 +10151,7 @@
       </c>
       <c r="G268" s="22" t="inlineStr">
         <is>
-          <t>Itération 8 — remboursement wallet intégral si payée</t>
+          <t>Itération 8 — remboursement wallet si payée (hors frais de service depuis le lot 3)</t>
         </is>
       </c>
     </row>
@@ -10741,7 +10741,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Frais de livraison par vendeur éditables, appliqués au panier et au checkout</t>
+          <t>Frais de livraison par vendeur, frais de service acheteur (%) et frais Mobile Money (%) éditables</t>
         </is>
       </c>
     </row>
@@ -14718,7 +14718,12 @@
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Lot 3 (2026-09-18) : demande de devis dans le chat, bon de commande vendeur (prix libres, livraison, validité), acceptation = commande avec paiement sécurisé, PDF proforma</t>
         </is>
       </c>
     </row>
@@ -22795,8 +22800,6 @@
         </is>
       </c>
     </row>
-    <row r="95"/>
-    <row r="96"/>
     <row r="97" ht="16.3" customHeight="1" s="26">
       <c r="A97" s="33" t="inlineStr">
         <is>
@@ -42326,7 +42329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="26" min="1" max="1"/>
@@ -43370,6 +43373,81 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Messagerie</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Bons de commande dans le chat : lignes catalogue ou libres, prix/livraison/validité libres, modification, refus motivé, expiration, PDF</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Lot 3 flux acheteur-vendeur (2026-09-18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Paiements</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Paiement depuis le chat : acceptation du bon, passage en caisse, carte « Payer maintenant »</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Lot 3 - sur wallet (mode démo), FedaPay à brancher</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Paiements</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Frais de service acheteur (1 %, non remboursables) + frais Mobile Money répercutés à la recharge, paramétrables</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Lot 3 - fonds sécurisés hors frais de service en admin</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
docs(suivi): MAJ Excel - recherche (MVP #76-77, Phase 2 #46-47, Phase 3 #18) + suivi technique
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -3920,7 +3920,7 @@
       </c>
       <c r="G82" s="22" t="inlineStr">
         <is>
-          <t>Itération 3 — dans l'en-tête du site</t>
+          <t>Itération 3 — dans l'en-tête ; lot 4 (2026-09-18) : autocomplétion produits/rayons/boutiques</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3955,7 @@
       </c>
       <c r="G83" s="22" t="inlineStr">
         <is>
-          <t>Itération 3 — titre + description</t>
+          <t>Lot 4 (2026-09-18) : plein texte français sans accents, synonymes, correction des fautes, rayons et boutiques, tri par pertinence</t>
         </is>
       </c>
     </row>
@@ -13739,7 +13739,12 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Lot 4 : suggestions au fil de la saisie (produits, rayons, boutiques), clavier, correction « Résultats pour … »</t>
         </is>
       </c>
     </row>
@@ -13769,7 +13774,12 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Lot 4 : tendances (30 j) dans la barre de recherche et en admin ; demandes non servies montrées aux vendeurs</t>
         </is>
       </c>
     </row>
@@ -20920,7 +20930,12 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Lot 4 : recherches récentes gardées sur l'appareil, proposées à l'ouverture de la barre</t>
         </is>
       </c>
     </row>
@@ -42329,7 +42344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="26" min="1" max="1"/>
@@ -43448,6 +43463,56 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Moteur plein texte PostgreSQL (tsvector français, unaccent, pg_trgm), synonymes éditables en admin, correction des fautes</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Lot 4 flux acheteur-vendeur (2026-09-18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Journal anonyme des recherches : tendances et demandes non servies (admin + tableau de bord vendeur)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Lot 4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
feat(medias): vidéo produit et téléchargement filigrané des médias
Lot 6 du flux acheteur-vendeur (docs/CHANGEMENTS.md §5).

Vidéo de présentation (migration 0023) : le vendeur téléverse un MP4, WebM
ou MOV de 60 s et 50 Mo maximum (durée vérifiée avant envoi), avec aperçu,
barre de progression, remplacement et retrait - l'ancien fichier est effacé
du stockage. La vidéo ouvre la galerie de la fiche et met une pastille de
lecture sur les cartes du catalogue.

Téléchargement des médias : /api/medias/[id] réservé aux comptes connectés
et aux fiches publiées. Les photos repartent filigranées « Deal Lomé »
(sharp : trame diagonale + bandeau titre/boutique/domaine) ; la vidéo est
servie en flux avec requêtes partielles, sans filigrane - la marquer
demanderait un ré-encodage ffmpeg sur le VPS.

Règles Storage : la vidéo (50 Mo) est autorisée sous products/{uid}/ à
côté des photos (5 Mo) - à republier au déploiement.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -3148,7 +3148,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>À faire</t>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Lot 6 : vidéo de présentation optionnelle (MP4/WebM/MOV, 60 s et 50 Mo max, durée vérifiée), affichée en tête de galerie et signalée par une pastille sur les cartes</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3188,7 @@
       </c>
       <c r="G60" s="22" t="inlineStr">
         <is>
-          <t>Itération 3</t>
+          <t>Itération 3 — aperçu des photos avant envoi ; lot 6 : aperçu de la vidéo avec lecteur</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3223,7 @@
       </c>
       <c r="G61" s="22" t="inlineStr">
         <is>
-          <t>Itération 3</t>
+          <t>Itération 3 — suppression des photos ; lot 6 : retrait/remplacement de la vidéo (ancien fichier effacé du stockage)</t>
         </is>
       </c>
     </row>
@@ -42479,7 +42484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="26" min="1" max="1"/>
@@ -43773,6 +43778,56 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Médias</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Vidéo de présentation produit : téléversement avec progression, contrôle de durée et de poids, lecture dans la galerie</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Lot 6 flux acheteur-vendeur (2026-09-21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Médias</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Téléchargement des médias réservé aux comptes connectés : photos filigranées « Deal Lomé » (sharp), vidéo en flux avec requêtes partielles</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Lot 6 - filigrane vidéo non couvert (ré-encodage ffmpeg)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>